<commit_message>
carga producto y modificacion completa
</commit_message>
<xml_diff>
--- a/NegocioFresa/recursos/fresa pagina RF_RNF.xlsx
+++ b/NegocioFresa/recursos/fresa pagina RF_RNF.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="90">
   <si>
     <t>ID</t>
   </si>
@@ -142,7 +142,46 @@
     <t>Registro de venta en tiempo real</t>
   </si>
   <si>
-    <t>Procesar la venta de productos, calculando el total y aplicando de forma inmediata el descuento del stock correspondiente en MySQL</t>
+    <t>Procesar la venta mediantes Transacciones Atómicas, registrando la cabecera (metodo de pago, usuario) y el detalle de los productos, aplicando el descuento de stock correspondiente en la base de datos SQLite.</t>
+  </si>
+  <si>
+    <t>RF 9.1</t>
+  </si>
+  <si>
+    <t>Búsqueda Dinámica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permitir la búsqueda y adición de productos al carrito mendiante escaneo de código de barras o panel de autocompletado por texto </t>
+  </si>
+  <si>
+    <t>RF 9.2</t>
+  </si>
+  <si>
+    <t>Ajustes y Descuentos Trazables</t>
+  </si>
+  <si>
+    <t>Permitir la palicación de descuentos o recargos manuales registrándolos como líneas independientes (tipo_linea) en el detalle de la venta, evitando la modificación manual y libre del precio final</t>
+  </si>
+  <si>
+    <t>RF 9.3</t>
+  </si>
+  <si>
+    <t>Medios de Pago e Impuestos</t>
+  </si>
+  <si>
+    <t>Registrar el método de pago utilizado (efectivo, mercado pago, etc) y calcular automáticamente recargos adicionales o impuestos, guardándolos en la cavecera de la venta</t>
+  </si>
+  <si>
+    <t>RF 9.4</t>
+  </si>
+  <si>
+    <t>Trazabilidad de Usuario</t>
+  </si>
+  <si>
+    <t>Vincular cada venta finalizada con el id_usuario que operó el sistema para audtoría interna</t>
+  </si>
+  <si>
+    <t>Altal</t>
   </si>
   <si>
     <t>RF 10</t>
@@ -202,13 +241,13 @@
     <t>RNF 2</t>
   </si>
   <si>
-    <t>main/flask</t>
+    <t>Tkinter de escritorio</t>
   </si>
   <si>
     <t>portabilidad</t>
   </si>
   <si>
-    <t>Acceso multidispositivo</t>
+    <t>Escritorio Local</t>
   </si>
   <si>
     <t>La interfaz de la página debe ser accesible desde computadoras y  teléfonos celulares de forma simultánea a través de la red local</t>
@@ -226,7 +265,7 @@
     <t>Persistencia relacional</t>
   </si>
   <si>
-    <t>Toda la información debe estar almacenada en un motor MySQL, asegurando que las modificaciones impacten inmediatamente y de forma segura</t>
+    <t>Toda la información debe estar almacenada en un motor SQLite, asegurando que las modificaciones impacten inmediatamente y de forma segura</t>
   </si>
   <si>
     <t>RNF 4</t>
@@ -1341,16 +1380,16 @@
         <v>44</v>
       </c>
       <c r="C12" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="F12" s="13" t="s">
         <v>46</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>48</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>11</v>
@@ -1378,19 +1417,19 @@
     <row r="13">
       <c r="A13" s="1"/>
       <c r="B13" s="12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>11</v>
@@ -1418,19 +1457,19 @@
     <row r="14">
       <c r="A14" s="1"/>
       <c r="B14" s="12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G14" s="14" t="s">
         <v>11</v>
@@ -1458,22 +1497,22 @@
     <row r="15">
       <c r="A15" s="1"/>
       <c r="B15" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F15" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E15" s="13" t="s">
+      <c r="G15" s="14" t="s">
         <v>56</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="G15" s="14" t="s">
-        <v>11</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -1498,13 +1537,13 @@
     <row r="16">
       <c r="A16" s="1"/>
       <c r="B16" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="D16" s="13" t="s">
         <v>59</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>8</v>
       </c>
       <c r="E16" s="13" t="s">
         <v>60</v>
@@ -1540,17 +1579,17 @@
       <c r="B17" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="F17" s="13" t="s">
         <v>64</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>66</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>11</v>
@@ -1578,19 +1617,19 @@
     <row r="18">
       <c r="A18" s="1"/>
       <c r="B18" s="12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>68</v>
+      <c r="C18" s="11" t="s">
+        <v>58</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G18" s="14" t="s">
         <v>11</v>
@@ -1618,19 +1657,19 @@
     <row r="19">
       <c r="A19" s="1"/>
       <c r="B19" s="12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="G19" s="14" t="s">
         <v>11</v>
@@ -1657,12 +1696,24 @@
     </row>
     <row r="20">
       <c r="A20" s="1"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="22"/>
+      <c r="B20" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>11</v>
+      </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -1685,12 +1736,24 @@
     </row>
     <row r="21">
       <c r="A21" s="1"/>
-      <c r="B21" s="19"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="22"/>
+      <c r="B21" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>11</v>
+      </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
@@ -1713,12 +1776,24 @@
     </row>
     <row r="22">
       <c r="A22" s="1"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="22"/>
+      <c r="B22" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G22" s="14" t="s">
+        <v>11</v>
+      </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -1741,12 +1816,24 @@
     </row>
     <row r="23">
       <c r="A23" s="1"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="22"/>
+      <c r="B23" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="G23" s="14" t="s">
+        <v>11</v>
+      </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
@@ -1853,12 +1940,12 @@
     </row>
     <row r="27">
       <c r="A27" s="1"/>
-      <c r="B27" s="23"/>
+      <c r="B27" s="19"/>
       <c r="C27" s="20"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="25"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="22"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
@@ -1881,12 +1968,12 @@
     </row>
     <row r="28">
       <c r="A28" s="1"/>
-      <c r="B28" s="23"/>
+      <c r="B28" s="19"/>
       <c r="C28" s="20"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="25"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="22"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
@@ -1909,12 +1996,12 @@
     </row>
     <row r="29">
       <c r="A29" s="1"/>
-      <c r="B29" s="23"/>
+      <c r="B29" s="19"/>
       <c r="C29" s="20"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="25"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="22"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
@@ -1937,12 +2024,12 @@
     </row>
     <row r="30">
       <c r="A30" s="1"/>
-      <c r="B30" s="26"/>
+      <c r="B30" s="19"/>
       <c r="C30" s="20"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="28"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="22"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
@@ -1965,12 +2052,12 @@
     </row>
     <row r="31">
       <c r="A31" s="1"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="31"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="25"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
@@ -1993,12 +2080,12 @@
     </row>
     <row r="32">
       <c r="A32" s="1"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="22"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="25"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
@@ -2021,12 +2108,12 @@
     </row>
     <row r="33">
       <c r="A33" s="1"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="22"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="25"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
@@ -2049,12 +2136,12 @@
     </row>
     <row r="34">
       <c r="A34" s="1"/>
-      <c r="B34" s="19"/>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="22"/>
+      <c r="B34" s="26"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="28"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
@@ -2077,12 +2164,12 @@
     </row>
     <row r="35">
       <c r="A35" s="1"/>
-      <c r="B35" s="19"/>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="22"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="30"/>
+      <c r="E35" s="30"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="31"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
@@ -2133,12 +2220,12 @@
     </row>
     <row r="37">
       <c r="A37" s="1"/>
-      <c r="B37" s="26"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="28"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="21"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="22"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
@@ -2161,12 +2248,12 @@
     </row>
     <row r="38">
       <c r="A38" s="1"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="22"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
@@ -2189,12 +2276,12 @@
     </row>
     <row r="39">
       <c r="A39" s="1"/>
-      <c r="B39" s="1"/>
-      <c r="C39" s="1"/>
-      <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="22"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
@@ -2217,12 +2304,12 @@
     </row>
     <row r="40">
       <c r="A40" s="1"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="21"/>
+      <c r="G40" s="22"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
       <c r="J40" s="1"/>
@@ -2245,12 +2332,12 @@
     </row>
     <row r="41">
       <c r="A41" s="1"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="28"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
@@ -29123,6 +29210,118 @@
       <c r="Y1000" s="1"/>
       <c r="Z1000" s="1"/>
     </row>
+    <row r="1001">
+      <c r="A1001" s="1"/>
+      <c r="B1001" s="1"/>
+      <c r="C1001" s="1"/>
+      <c r="D1001" s="1"/>
+      <c r="E1001" s="1"/>
+      <c r="F1001" s="1"/>
+      <c r="G1001" s="1"/>
+      <c r="H1001" s="1"/>
+      <c r="I1001" s="1"/>
+      <c r="J1001" s="1"/>
+      <c r="K1001" s="1"/>
+      <c r="L1001" s="1"/>
+      <c r="M1001" s="1"/>
+      <c r="N1001" s="1"/>
+      <c r="O1001" s="1"/>
+      <c r="P1001" s="1"/>
+      <c r="Q1001" s="1"/>
+      <c r="R1001" s="1"/>
+      <c r="S1001" s="1"/>
+      <c r="T1001" s="1"/>
+      <c r="U1001" s="1"/>
+      <c r="V1001" s="1"/>
+      <c r="W1001" s="1"/>
+      <c r="X1001" s="1"/>
+      <c r="Y1001" s="1"/>
+      <c r="Z1001" s="1"/>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="1"/>
+      <c r="B1002" s="1"/>
+      <c r="C1002" s="1"/>
+      <c r="D1002" s="1"/>
+      <c r="E1002" s="1"/>
+      <c r="F1002" s="1"/>
+      <c r="G1002" s="1"/>
+      <c r="H1002" s="1"/>
+      <c r="I1002" s="1"/>
+      <c r="J1002" s="1"/>
+      <c r="K1002" s="1"/>
+      <c r="L1002" s="1"/>
+      <c r="M1002" s="1"/>
+      <c r="N1002" s="1"/>
+      <c r="O1002" s="1"/>
+      <c r="P1002" s="1"/>
+      <c r="Q1002" s="1"/>
+      <c r="R1002" s="1"/>
+      <c r="S1002" s="1"/>
+      <c r="T1002" s="1"/>
+      <c r="U1002" s="1"/>
+      <c r="V1002" s="1"/>
+      <c r="W1002" s="1"/>
+      <c r="X1002" s="1"/>
+      <c r="Y1002" s="1"/>
+      <c r="Z1002" s="1"/>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="1"/>
+      <c r="B1003" s="1"/>
+      <c r="C1003" s="1"/>
+      <c r="D1003" s="1"/>
+      <c r="E1003" s="1"/>
+      <c r="F1003" s="1"/>
+      <c r="G1003" s="1"/>
+      <c r="H1003" s="1"/>
+      <c r="I1003" s="1"/>
+      <c r="J1003" s="1"/>
+      <c r="K1003" s="1"/>
+      <c r="L1003" s="1"/>
+      <c r="M1003" s="1"/>
+      <c r="N1003" s="1"/>
+      <c r="O1003" s="1"/>
+      <c r="P1003" s="1"/>
+      <c r="Q1003" s="1"/>
+      <c r="R1003" s="1"/>
+      <c r="S1003" s="1"/>
+      <c r="T1003" s="1"/>
+      <c r="U1003" s="1"/>
+      <c r="V1003" s="1"/>
+      <c r="W1003" s="1"/>
+      <c r="X1003" s="1"/>
+      <c r="Y1003" s="1"/>
+      <c r="Z1003" s="1"/>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="1"/>
+      <c r="B1004" s="1"/>
+      <c r="C1004" s="1"/>
+      <c r="D1004" s="1"/>
+      <c r="E1004" s="1"/>
+      <c r="F1004" s="1"/>
+      <c r="G1004" s="1"/>
+      <c r="H1004" s="1"/>
+      <c r="I1004" s="1"/>
+      <c r="J1004" s="1"/>
+      <c r="K1004" s="1"/>
+      <c r="L1004" s="1"/>
+      <c r="M1004" s="1"/>
+      <c r="N1004" s="1"/>
+      <c r="O1004" s="1"/>
+      <c r="P1004" s="1"/>
+      <c r="Q1004" s="1"/>
+      <c r="R1004" s="1"/>
+      <c r="S1004" s="1"/>
+      <c r="T1004" s="1"/>
+      <c r="U1004" s="1"/>
+      <c r="V1004" s="1"/>
+      <c r="W1004" s="1"/>
+      <c r="X1004" s="1"/>
+      <c r="Y1004" s="1"/>
+      <c r="Z1004" s="1"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C3"/>
@@ -29139,8 +29338,12 @@
     <hyperlink r:id="rId12" ref="C14"/>
     <hyperlink r:id="rId13" ref="C15"/>
     <hyperlink r:id="rId14" ref="C16"/>
-    <hyperlink r:id="rId15" ref="C19"/>
+    <hyperlink r:id="rId15" ref="C17"/>
+    <hyperlink r:id="rId16" ref="C18"/>
+    <hyperlink r:id="rId17" ref="C19"/>
+    <hyperlink r:id="rId18" ref="C20"/>
+    <hyperlink r:id="rId19" ref="C23"/>
   </hyperlinks>
-  <drawing r:id="rId16"/>
+  <drawing r:id="rId20"/>
 </worksheet>
 </file>
</xml_diff>